<commit_message>
ADD: all 5 exercises of KC#5 completed and verified
</commit_message>
<xml_diff>
--- a/data/registration-data.xlsx
+++ b/data/registration-data.xlsx
@@ -430,7 +430,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>R01</v>
+        <v>REG_VAL01</v>
       </c>
       <c r="B2" t="str">
         <v>Valid short names with mixed-case password</v>
@@ -451,7 +451,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H2" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -459,7 +459,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>R02</v>
+        <v>REG_VAL02</v>
       </c>
       <c r="B3" t="str">
         <v>Valid hyphenated username slug</v>
@@ -480,7 +480,7 @@
         <v>abc1234</v>
       </c>
       <c r="H3" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -488,7 +488,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>R03</v>
+        <v>REG_VAL03</v>
       </c>
       <c r="B4" t="str">
         <v>Valid registration with numeric-heavy password</v>
@@ -509,7 +509,7 @@
         <v>1234abcd</v>
       </c>
       <c r="H4" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -517,7 +517,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>R04</v>
+        <v>REG_VAL04</v>
       </c>
       <c r="B5" t="str">
         <v>Valid registration with symbol-rich password</v>
@@ -538,7 +538,7 @@
         <v>P@ss!2024</v>
       </c>
       <c r="H5" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -546,7 +546,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>R05</v>
+        <v>REG_VAL05</v>
       </c>
       <c r="B6" t="str">
         <v>Valid registration near max username length</v>
@@ -567,7 +567,7 @@
         <v>Secure99!</v>
       </c>
       <c r="H6" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -575,7 +575,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>R06</v>
+        <v>REG_EMAIL01</v>
       </c>
       <c r="B7" t="str">
         <v>Invalid email shape: missing @ symbol</v>
@@ -596,7 +596,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H7" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -604,7 +604,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>R07</v>
+        <v>REG_EMAIL02</v>
       </c>
       <c r="B8" t="str">
         <v>Invalid email shape: multiple @ symbols</v>
@@ -625,7 +625,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H8" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I8" t="str">
         <v>Invalid username. Usernames can only contain lowercase letters, numbers, and single hyphens, must be between 3 and 39 characters, and cannot start or end with a hyphen.</v>
@@ -633,7 +633,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>R08</v>
+        <v>REG_EMAIL03</v>
       </c>
       <c r="B9" t="str">
         <v>Invalid email shape: no domain after @</v>
@@ -654,7 +654,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H9" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I9" t="str">
         <v>Invalid username. Usernames can only contain lowercase letters, numbers, and single hyphens, must be between 3 and 39 characters, and cannot start or end with a hyphen.</v>
@@ -662,7 +662,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>R09</v>
+        <v>REG_EMAIL04</v>
       </c>
       <c r="B10" t="str">
         <v>Invalid email shape: no TLD</v>
@@ -683,7 +683,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H10" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I10" t="str">
         <v>Invalid username. Usernames can only contain lowercase letters, numbers, and single hyphens, must be between 3 and 39 characters, and cannot start or end with a hyphen.</v>
@@ -691,7 +691,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>R10</v>
+        <v>REG_EMAIL05</v>
       </c>
       <c r="B11" t="str">
         <v>Invalid email shape: spaces in address</v>
@@ -712,7 +712,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H11" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I11" t="str">
         <v>Invalid username. Usernames can only contain lowercase letters, numbers, and single hyphens, must be between 3 and 39 characters, and cannot start or end with a hyphen.</v>
@@ -720,7 +720,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>R11</v>
+        <v>REG_MISMATCH01</v>
       </c>
       <c r="B12" t="str">
         <v>Password mismatch: trailing digit differs</v>
@@ -741,7 +741,7 @@
         <v>Passw0rd1!</v>
       </c>
       <c r="H12" t="str">
-        <v>mismatch</v>
+        <v>fail</v>
       </c>
       <c r="I12" t="str">
         <v>Passwords do not match.</v>
@@ -749,7 +749,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>R12</v>
+        <v>REG_MISMATCH02</v>
       </c>
       <c r="B13" t="str">
         <v>Password mismatch: case difference only</v>
@@ -770,7 +770,7 @@
         <v>passw0rd!</v>
       </c>
       <c r="H13" t="str">
-        <v>mismatch</v>
+        <v>fail</v>
       </c>
       <c r="I13" t="str">
         <v>Passwords do not match.</v>
@@ -778,7 +778,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>R13</v>
+        <v>REG_MISMATCH03</v>
       </c>
       <c r="B14" t="str">
         <v>Password mismatch: completely different confirm value</v>
@@ -799,7 +799,7 @@
         <v>Different1!</v>
       </c>
       <c r="H14" t="str">
-        <v>mismatch</v>
+        <v>fail</v>
       </c>
       <c r="I14" t="str">
         <v>Passwords do not match.</v>
@@ -807,7 +807,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>R14</v>
+        <v>REG_LEN01</v>
       </c>
       <c r="B15" t="str">
         <v>Password length boundary: min minus 1 (3 chars)</v>
@@ -828,7 +828,7 @@
         <v>abc</v>
       </c>
       <c r="H15" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I15" t="str">
         <v>Password must be at least 4 characters long.</v>
@@ -836,7 +836,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>R15</v>
+        <v>REG_LEN02</v>
       </c>
       <c r="B16" t="str">
         <v>Password length boundary: minimum (4 chars)</v>
@@ -857,7 +857,7 @@
         <v>abcd</v>
       </c>
       <c r="H16" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -865,7 +865,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>R16</v>
+        <v>REG_LEN03</v>
       </c>
       <c r="B17" t="str">
         <v>Password length boundary: long password (65 chars)</v>
@@ -886,7 +886,7 @@
         <v>aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</v>
       </c>
       <c r="H17" t="str">
-        <v>success</v>
+        <v>pass</v>
       </c>
       <c r="I17" t="str">
         <v/>
@@ -894,7 +894,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>R17</v>
+        <v>REG_REQ01</v>
       </c>
       <c r="B18" t="str">
         <v>Missing required field: blank username</v>
@@ -915,7 +915,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H18" t="str">
-        <v>required</v>
+        <v>fail</v>
       </c>
       <c r="I18" t="str">
         <v>All fields are required.</v>
@@ -923,7 +923,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>R18</v>
+        <v>REG_REQ02</v>
       </c>
       <c r="B19" t="str">
         <v>Missing required field: blank password</v>
@@ -944,7 +944,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H19" t="str">
-        <v>required</v>
+        <v>fail</v>
       </c>
       <c r="I19" t="str">
         <v>All fields are required.</v>
@@ -952,7 +952,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>R19</v>
+        <v>REG_SPEC01</v>
       </c>
       <c r="B20" t="str">
         <v>Special char in name: apostrophe in first name</v>
@@ -973,7 +973,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H20" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I20" t="str">
         <v>Invalid username. Usernames can only contain lowercase letters, numbers, and single hyphens, must be between 3 and 39 characters, and cannot start or end with a hyphen.</v>
@@ -981,7 +981,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>R20</v>
+        <v>REG_SPEC02</v>
       </c>
       <c r="B21" t="str">
         <v>Special char in name: accented chars and emoji</v>
@@ -1002,7 +1002,7 @@
         <v>Passw0rd!</v>
       </c>
       <c r="H21" t="str">
-        <v>error</v>
+        <v>fail</v>
       </c>
       <c r="I21" t="str">
         <v>Invalid username. Usernames can only contain lowercase letters, numbers, and single hyphens, must be between 3 and 39 characters, and cannot start or end with a hyphen.</v>

</xml_diff>